<commit_message>
Add postfix run1 audit results - first audit_result finding
</commit_message>
<xml_diff>
--- a/results/audit_results.xlsx
+++ b/results/audit_results.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="pacemaker_run2_advisory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="postfix_run1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -950,4 +951,981 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>--- application ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>is_app</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>is_library</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>postfix/src/anvil</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>The 'anvil' component in Postfix serves as a connection count and rate limiter daemon, helping manage and restrict connections to the mail system.The 'anvil' component in Postfix serves as a connection count and rate limiter daemon, helping manage and restrict connections to the mail system.</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>postfix/src/bounce</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>The 'bounce' component handles bounced or deferred emails in the Postfix mail system.The 'bounce' component handles bounced or deferred emails in the Postfix mail system.The 'bounce' component handles bounced or deferred emails in the Postfix mail system.The 'bounce' component handles bounced or deferred emails in the Postfix mail system.</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>postfix/src/cleanup</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>postfix/src/discard</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>The 'discard' component is a trivial discard mailer in the Postfix mail system, used to intentionally discard messages.The 'discard' component is a trivial discard mailer in the Postfix mail system, used to intentionally discard messages.The 'discard' component is a trivial discard mailer in the Postfix mail system, used to intentionally discard messages.The 'discard' component is a trivial discard mailer in the Postfix mail system, used to intentionally discard messages.</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>postfix/src/local</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>The 'local' component handles the local delivery of emails in the Postfix mail system.The 'local' component handles the local delivery of emails in the Postfix mail system.</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>postfix/src/master</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>The 'master' component is the core Postfix super-server daemon that manages all mail-related processes.</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>..</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>--- entry_point ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>user_input</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>app_id</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>postfix/src/anvil/anvil.c</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>argc, argv</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1026</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>The main function is the entry point of the 'anvil' application. Here, argc and argv represent user-supplied arguments to the program. While configuration files or predefined inputs are trusted, user-supplied arguments are treated as potentially untrusted inputs due to the possibility of pointing to dubious resources or being subject to manipulation.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>postfix/src/discard/discard.c</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>argc, argv</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>243</v>
+      </c>
+      <c r="E16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>The 'main' function is an entry point to the discard service. It passes control to the single-threaded skeleton function 'single_server_main', which executes with the 'discard_service'. The application's main function parameters, 'argc' and 'argv', can potentially include user-supplied data when launching the application. These inputs are considered untrusted and could pose risks if not properly validated or sanitized.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>postfix/src/cleanup/cleanup.c</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>src</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>547</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>The 'cleanup_service' function processes incoming mail messages, exposing them to the application. The 'src' input is considered untrusted as it comes from external sources, potentially containing user-generated email payloads.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>postfix/src/cleanup/cleanup.c</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>argv</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>665</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>The 'main' function initializes and passes control to the single-threaded service skeleton. User inputs via 'argv' are validated to ensure there are no command-line arguments that can introduce anomalies.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>--- user_action ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>app_id</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>postfix/src/discard/discard.c</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>207</v>
+      </c>
+      <c r="E22" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>The function `discard_service` processes client connections to the discard mailer via a UNIX-domain socket. It reads delivery requests and subsequently processes those intended for discard. Users are allowed to issue delivery requests via the queue manager, with messages ultimately discarded as intended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>postfix/src/smtpd/smtpd.c</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>237</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>This section of code defines the default action and behavior for Milter (mail filter) responses when they are unavailable. It specifies actions for interacting with mail filter applications, including handling SMTP commands and defining behavior on failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>--- application_issue ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>component_id</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Input Handling Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>The component handles bounced or deferred emails and may involve processing untrusted email and header content. Risks include injection vulnerabilities and improper handling of malformed email data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Inter-module Communication Risks</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>The component likely interacts with other modules or external email servers via network protocols like SMTP or filesystem operations, which may include potential risks in privilege escalation or injection attacks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Injection Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Mail systems frequently process untrusted user input, which could result in risks like header injection, command injection, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>4</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Authentication and Authorization Logic</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>As the system includes authentication mechanisms, there is potential for bypass or mismanagement of access control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Injection via Email Content</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>The component processes incoming mail messages and user-generated payloads. High risk exists for injection attacks through email headers or body content that exploit weak validation or insufficient canonicalization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Encryption and Transmission Security</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Handling TLS encryption and sensitive email data during transfer introduces risk factors for confidentiality breaches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>7</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Buffer Overflow or Memory Mismanagement</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Handling large volumes of emails or malicious payloads could lead to buffer overflows, especially given unknown or untrusted inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>8</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>8</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Protocol Security Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>The component implements authentication protocols (SASL) and encryption mechanisms (TLS). Improper implementation could result in authentication bypass, weak encryption, or exploitation of these protocols, exposing data to attackers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>9</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>8</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Email-Based Input Risks</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Email filter and processing mechanisms may be prone to spam, phishing, or injection attacks. Untrusted email inputs could bypass the filters and lead to malicious mail delivery or system exploit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>10</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Improper Error Handling Risks</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Failure to handle malformed email inputs or invalid protocol data appropriately may lead to system instability, denial of service, or crash scenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>--- web_entry_point ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>middleware</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>roles_scopes</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>entry_point_id</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>--- audit_result ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>component_id</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>issue_id</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>has_vulnerability</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>has_non_security_error</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Improper Error Handling Risks</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>10</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Audit focused on whether malformed email inputs or invalid protocol data lead to system faults or crash scenarios. Explored the SMTP daemon (postfix/src/smtpd/smtpd.c), focused on error-class handler mechanisms (e.g., 4XX/5XX responses). Identified programmatic containment of such errors, with no exploitable scenarios or vulnerabilities detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>--- low_severity_audit_result ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>component_id</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>result_id</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rerun using known application issues to find more audits
</commit_message>
<xml_diff>
--- a/results/audit_results.xlsx
+++ b/results/audit_results.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="pacemaker_run2_advisory" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="postfix_run1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="postfix_run2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1010,7 +1011,6 @@
           <t>vdukhovni/postfix</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).</t>
@@ -1920,6 +1920,1123 @@
         </is>
       </c>
       <c r="E46" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>--- application ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>is_app</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>is_library</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>postfix/src/anvil</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>The 'anvil' component in Postfix serves as a connection count and rate limiter daemon, helping manage and restrict connections to the mail system.The 'anvil' component in Postfix serves as a connection count and rate limiter daemon, helping manage and restrict connections to the mail system.</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>postfix/src/bounce</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>The 'bounce' component handles bounced or deferred emails in the Postfix mail system.The 'bounce' component handles bounced or deferred emails in the Postfix mail system.The 'bounce' component handles bounced or deferred emails in the Postfix mail system.The 'bounce' component handles bounced or deferred emails in the Postfix mail system.</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>postfix/src/cleanup</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.The 'cleanup' component is responsible for canonicalizing and enqueuing mail in the Postfix mail system.</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>postfix/src/discard</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>The 'discard' component is a trivial discard mailer in the Postfix mail system, used to intentionally discard messages.The 'discard' component is a trivial discard mailer in the Postfix mail system, used to intentionally discard messages.The 'discard' component is a trivial discard mailer in the Postfix mail system, used to intentionally discard messages.The 'discard' component is a trivial discard mailer in the Postfix mail system, used to intentionally discard messages.</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>postfix/src/local</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>The 'local' component handles the local delivery of emails in the Postfix mail system.The 'local' component handles the local delivery of emails in the Postfix mail system.</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>postfix/src/master</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>The 'master' component is the core Postfix super-server daemon that manages all mail-related processes.</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>..</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).The Postfix repository is a mail system library and framework. It serves as a robust, secure, and flexible alternative to the sendmail program. The library provides essential functionality to manage and transfer emails, supporting mail filters, authentication protocols (SASL), and encryption (TLS).</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>--- entry_point ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>user_input</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>app_id</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>postfix/src/anvil/anvil.c</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>argc, argv</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1026</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>The main function is the entry point of the 'anvil' application. Here, argc and argv represent user-supplied arguments to the program. While configuration files or predefined inputs are trusted, user-supplied arguments are treated as potentially untrusted inputs due to the possibility of pointing to dubious resources or being subject to manipulation.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>postfix/src/discard/discard.c</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>argc, argv</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>243</v>
+      </c>
+      <c r="E16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>The 'main' function is an entry point to the discard service. It passes control to the single-threaded skeleton function 'single_server_main', which executes with the 'discard_service'. The application's main function parameters, 'argc' and 'argv', can potentially include user-supplied data when launching the application. These inputs are considered untrusted and could pose risks if not properly validated or sanitized.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>postfix/src/cleanup/cleanup.c</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>src</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>547</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>The 'cleanup_service' function processes incoming mail messages, exposing them to the application. The 'src' input is considered untrusted as it comes from external sources, potentially containing user-generated email payloads.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>postfix/src/cleanup/cleanup.c</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>argv</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>665</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>The 'main' function initializes and passes control to the single-threaded service skeleton. User inputs via 'argv' are validated to ensure there are no command-line arguments that can introduce anomalies.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>--- user_action ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>app_id</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>postfix/src/discard/discard.c</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>207</v>
+      </c>
+      <c r="E22" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>The function `discard_service` processes client connections to the discard mailer via a UNIX-domain socket. It reads delivery requests and subsequently processes those intended for discard. Users are allowed to issue delivery requests via the queue manager, with messages ultimately discarded as intended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>postfix/src/smtpd/smtpd.c</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>237</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>This section of code defines the default action and behavior for Milter (mail filter) responses when they are unavailable. It specifies actions for interacting with mail filter applications, including handling SMTP commands and defining behavior on failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>--- application_issue ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>component_id</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Input Handling Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>The component handles bounced or deferred emails and may involve processing untrusted email and header content. Risks include injection vulnerabilities and improper handling of malformed email data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Inter-module Communication Risks</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>The component likely interacts with other modules or external email servers via network protocols like SMTP or filesystem operations, which may include potential risks in privilege escalation or injection attacks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Injection Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Mail systems frequently process untrusted user input, which could result in risks like header injection, command injection, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>4</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Authentication and Authorization Logic</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>As the system includes authentication mechanisms, there is potential for bypass or mismanagement of access control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Injection via Email Content</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>The component processes incoming mail messages and user-generated payloads. High risk exists for injection attacks through email headers or body content that exploit weak validation or insufficient canonicalization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Encryption and Transmission Security</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Handling TLS encryption and sensitive email data during transfer introduces risk factors for confidentiality breaches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>7</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Buffer Overflow or Memory Mismanagement</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Handling large volumes of emails or malicious payloads could lead to buffer overflows, especially given unknown or untrusted inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>8</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>8</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Protocol Security Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>The component implements authentication protocols (SASL) and encryption mechanisms (TLS). Improper implementation could result in authentication bypass, weak encryption, or exploitation of these protocols, exposing data to attackers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>9</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>8</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Email-Based Input Risks</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Email filter and processing mechanisms may be prone to spam, phishing, or injection attacks. Untrusted email inputs could bypass the filters and lead to malicious mail delivery or system exploit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>10</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Improper Error Handling Risks</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Failure to handle malformed email inputs or invalid protocol data appropriately may lead to system instability, denial of service, or crash scenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>--- web_entry_point ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>middleware</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>roles_scopes</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>entry_point_id</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>--- audit_result ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>component_id</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>issue_id</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>has_vulnerability</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>has_non_security_error</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Improper Error Handling Risks</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>10</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Audit focused on whether malformed email inputs or invalid protocol data lead to system faults or crash scenarios. Explored the SMTP daemon (postfix/src/smtpd/smtpd.c), focused on error-class handler mechanisms (e.g., 4XX/5XX responses). Identified programmatic containment of such errors, with no exploitable scenarios or vulnerabilities detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>3</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Inter-module Communication Risks</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>The analysis of the 'bounce.c' file confirms no exploitable inter-module communication vulnerabilities. All user inputs and inter-module data exchanges undergo stringent validation and sanitization to avoid risks such as privilege escalation or injection attacks. Observed functionality aligns with intended operations of handling bounced or deferred emails in Postfix. No further security concerns were identified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>3</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Input Handling Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>The audit revealed potential injection vulnerabilities through insufficient sanitization of queue IDs and queue names. Specific lines in postfix/src/bounce/bounce.c (lines: 282, 282) validate input but leave some gap for crafted malicious payloads. Memory corruption risks due to mishandling of buffers were observed, and addressable security enhancements for input sanitization are recommended.The audit concluded that the "bounce" component of the Postfix mail system correctly handles input validation and sanitization for bounced or deferred emails. Functions such as bounce_append_proto, bounce_notify_proto, bounce_verp_proto, and bounce_one_proto implement mechanisms to validate and sanitize user-controlled inputs (e.g., queue ID, queue name, sender, etc.). This includes using functions like mail_queue_id_ok, mail_queue_name_ok, and VS_NEUTER for strict input sanitization. Besides, malformed inputs are flagged with warnings or errors, and cleanup mechanisms are in place to mitigate risks. No vulnerabilities were identified, and input-handling protections were deemed adequate to address potential injection or data-malformation risks. Further security hardening through standard input validation libraries and additional tests are recommended but not indicative of a vulnerability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>4</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Injection via Email Content</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Audit Findings:
+1. **Validation in Cleanup Service**:
+   - Strict validation with `ATTR_FLAG_STRICT` ensures client processing options are correctly parsed.
+   - Safeguard mechanisms prevent the injection of hidden or malformed record types (e.g., record type checks and cleanup validation).
+2. **Sanitization of Records and Headers**:
+   - Incoming headers are transformed appropriately using routines and configurable tables.
+   - Functional reliance on external systems like `trivial-rewrite(8)` and Milter protocols for broader configuration and sanitization.
+3. **Potential Concerns**:
+   - Parsing mechanisms rely on external configurations such as `header_checks`, `body_checks`, and Milter protocols, which could be exploited in case of misconfiguration.
+4. **Conclusion**:
+   - No vulnerabilities identified within the `cleanup` component. Proper validation mechanisms prevent injection attacks through malformed headers or bodies.
+   - Recommendations: Ensure strict configuration of external sanitization settings like `header_checks` and `body_checks`.
+This concludes the audit for issue ID 5 in repo `vdukhovni/postfix`. No vulnerabilities confirmed; no security-related bugs found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>5</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>vdukhovni/postfix</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Buffer Overflow or Memory Mismanagement</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>7</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Audit revealed no direct misuse or lack of checks exposing buffer overflow vulnerabilities. Error handling related to excessive file sizes is partially managed (e.g., EFBIG in cleanup_out.c). Safeguards against buffer interactions with untrusted inputs remain insufficiently defined in some cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>--- low_severity_audit_result ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>component_id</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>result_id</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>reason</t>
         </is>

</xml_diff>